<commit_message>
scan: seg2 2026-06-22 21:31 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq3_2026-06-22.xlsx
+++ b/output/full_scan/batch_seq3_2026-06-22.xlsx
@@ -538,7 +538,7 @@
         <v/>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1300.431624199344</v>
+        <v>1310.431624199344</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>339</v>
@@ -580,21 +580,21 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>2458</v>
+        <v>2498</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>義隆</t>
+          <t>宏達電</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
         <v/>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1214.4423868037</v>
+        <v>1231.449113351784</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>178.5</v>
+        <v>50.4</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -605,16 +605,16 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>69.38785042652614</v>
+        <v>62.79255456154838</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>21.04057856850219</v>
+        <v>21.85446877541005</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>2.658968396144593</v>
+        <v>1.9111618683881</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L3" s="2" t="n">
         <v>0</v>
@@ -623,31 +623,31 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>1.045854883485862</v>
+        <v>0.2957715394739644</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, hist_turn_positive, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>2498</v>
+        <v>2458</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>宏達電</t>
+          <t>義隆</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
         <v/>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1211.449113351784</v>
+        <v>1214.4423868037</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>50.4</v>
+        <v>178.5</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -658,16 +658,16 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>62.79255456154838</v>
+        <v>69.38785042652614</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>21.85446877541005</v>
+        <v>21.04057856850219</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>1.9111618683881</v>
+        <v>2.658968396144593</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>0</v>
@@ -676,11 +676,11 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.2957715394739644</v>
+        <v>1.045854883485862</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, hist_turn_positive, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1191.144800504456</v>
+        <v>1201.144800504456</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>567</v>
@@ -750,7 +750,7 @@
         <v/>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1178.455065930137</v>
+        <v>1163.455065930137</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>176</v>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1126.67295722934</v>
+        <v>1136.67295722934</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>173.5</v>
@@ -1110,21 +1110,21 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>3041</v>
+        <v>3015</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>揚智</t>
+          <t>全漢</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1040.821337545846</v>
+        <v>1041.128635113892</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>30.95</v>
+        <v>65.8</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1135,13 +1135,13 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>70.38818322834021</v>
+        <v>65.04336866850539</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>22.25473792663648</v>
+        <v>27.933603229631</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>2.227575607681159</v>
+        <v>1.732179926346756</v>
       </c>
       <c r="K13" s="2" t="n">
         <v>2</v>
@@ -1153,31 +1153,31 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.535250857468736</v>
+        <v>0.2467961234320865</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>3015</v>
+        <v>3041</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>全漢</t>
+          <t>揚智</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1031.128635113892</v>
+        <v>1040.821337545846</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>65.8</v>
+        <v>30.95</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -1188,13 +1188,13 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>65.04336866850539</v>
+        <v>70.38818322834021</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>27.933603229631</v>
+        <v>22.25473792663648</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>1.732179926346756</v>
+        <v>2.227575607681159</v>
       </c>
       <c r="K14" s="2" t="n">
         <v>2</v>
@@ -1206,11 +1206,11 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.2467961234320865</v>
+        <v>0.535250857468736</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -1746,21 +1746,21 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>3023</v>
+        <v>3092</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>信邦</t>
+          <t>鴻碩</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>892.3468518390598</v>
+        <v>898.097008493026</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>333</v>
+        <v>32.7</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1771,16 +1771,16 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>61.65381114421583</v>
+        <v>59.86218099800117</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>18.14271909073128</v>
+        <v>17.44194148538615</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>1.023669751191906</v>
+        <v>2.355460889949802</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>0</v>
@@ -1789,31 +1789,31 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-0.00287829572828</v>
+        <v>0.3743764176286798</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, foreign_buy_3d, obv_uptrend, dealer_buy_3d, bb_squeeze_breakout, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, stronger_than_market, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>3092</v>
+        <v>3023</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>鴻碩</t>
+          <t>信邦</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>888.097008493026</v>
+        <v>892.3468518390598</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>32.7</v>
+        <v>333</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1824,16 +1824,16 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>59.86218099800117</v>
+        <v>61.65381114421583</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>17.44194148538615</v>
+        <v>18.14271909073128</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>2.355460889949802</v>
+        <v>1.023669751191906</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L26" s="2" t="n">
         <v>0</v>
@@ -1842,31 +1842,31 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.3743764176286798</v>
+        <v>-0.00287829572828</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, stronger_than_market, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, foreign_buy_3d, obv_uptrend, dealer_buy_3d, bb_squeeze_breakout, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>2890</v>
+        <v>2489</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>永豐金</t>
+          <t>瑞軒</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>884.6813077376228</v>
+        <v>890.8382474817712</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>39.8</v>
+        <v>50.7</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1877,49 +1877,49 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>81.08551076471412</v>
+        <v>59.84202454266753</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>38.7035707556817</v>
+        <v>14.70686052724877</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>1.568130773762281</v>
+        <v>1.481044188872043</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M27" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.8070011048307479</v>
+        <v>0.2071112357654536</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>3014</v>
+        <v>2890</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>聯陽</t>
+          <t>永豐金</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>884.5458553230603</v>
+        <v>884.6813077376228</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>160.5</v>
+        <v>39.8</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,49 +1930,49 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>66.84544922971048</v>
+        <v>81.08551076471412</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>39.22974043444355</v>
+        <v>38.7035707556817</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.9739038832140112</v>
+        <v>1.568130773762281</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M28" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.554674811267903</v>
+        <v>0.8070011048307479</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>2489</v>
+        <v>3014</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>瑞軒</t>
+          <t>聯陽</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>880.8382474817712</v>
+        <v>884.5458553230603</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>50.7</v>
+        <v>160.5</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,29 +1983,29 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>59.84202454266753</v>
+        <v>66.84544922971048</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>14.70686052724877</v>
+        <v>39.22974043444355</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>1.481044188872043</v>
+        <v>0.9739038832140112</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M29" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.2071112357654536</v>
+        <v>0.554674811267903</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -2075,7 +2075,7 @@
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>863.6796225933366</v>
+        <v>873.6796225933366</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>82.5</v>
@@ -2117,21 +2117,21 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>3004</v>
+        <v>2467</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>豐達科</t>
+          <t>志聖</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>862.139317117456</v>
+        <v>859.6113826937179</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>138</v>
+        <v>630</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,49 +2142,49 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>60.29043415428433</v>
+        <v>58.35777664589644</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>27.35039989787189</v>
+        <v>17.23562799992765</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.5139317117455965</v>
+        <v>0.8021939969537175</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M32" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.3750794643427864</v>
+        <v>0.3419759811628102</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>2467</v>
+        <v>3004</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>志聖</t>
+          <t>豐達科</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>859.6113826937179</v>
+        <v>852.139317117456</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>630</v>
+        <v>138</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,29 +2195,29 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>58.35777664589644</v>
+        <v>60.29043415428433</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>17.23562799992765</v>
+        <v>27.35039989787189</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.8021939969537175</v>
+        <v>0.5139317117455965</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M33" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.3419759811628102</v>
+        <v>0.3750794643427864</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -2329,21 +2329,21 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>3066</v>
+        <v>2832</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>李洲</t>
+          <t>台產</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>835.5541265731346</v>
+        <v>841.6013783667249</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>22.05</v>
+        <v>56.5</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2354,16 +2354,16 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>58.65694701105082</v>
+        <v>62.4807541109329</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>25.66316937847985</v>
+        <v>31.64023501447944</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>0.846245104721226</v>
+        <v>1.57437691944485</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L36" s="2" t="n">
         <v>0</v>
@@ -2372,31 +2372,31 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.0281983948711611</v>
+        <v>0.1296658344093935</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>3044</v>
+        <v>3066</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>健鼎</t>
+          <t>李洲</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>832.4412108981775</v>
+        <v>835.5541265731346</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>566</v>
+        <v>22.05</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,16 +2407,16 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>65.60254738701281</v>
+        <v>58.65694701105082</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>26.31960765830754</v>
+        <v>25.66316937847985</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0.7130586144020776</v>
+        <v>0.846245104721226</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L37" s="2" t="n">
         <v>0</v>
@@ -2425,31 +2425,31 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>6.027378470387969</v>
+        <v>-0.0281983948711611</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>2832</v>
+        <v>3044</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>台產</t>
+          <t>健鼎</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>831.6013783667249</v>
+        <v>832.4412108981775</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>56.5</v>
+        <v>566</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,16 +2460,16 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>62.4807541109329</v>
+        <v>65.60254738701281</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>31.64023501447944</v>
+        <v>26.31960765830754</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>1.57437691944485</v>
+        <v>0.7130586144020776</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L38" s="2" t="n">
         <v>0</v>
@@ -2478,11 +2478,11 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.1296658344093935</v>
+        <v>6.027378470387969</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -2647,41 +2647,41 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>2888</v>
+        <v>3059</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>新光金</t>
+          <t>華晶科</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>803.734991423423</v>
+        <v>804.0157793709948</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>12.05</v>
+        <v>49.35</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G42" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>56.43248093998274</v>
+        <v>61.30021418096327</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>29.57807013660666</v>
+        <v>35.72012135730295</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.1734991423423021</v>
+        <v>0.4943148480157628</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>0</v>
@@ -2690,51 +2690,51 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.0017859086290685</v>
+        <v>0.008391466478546401</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>3088</v>
+        <v>2888</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>艾訊</t>
+          <t>新光金</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>791.5428041139836</v>
+        <v>803.734991423423</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>144</v>
+        <v>12.05</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="G43" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>61.03457006201996</v>
+        <v>56.43248093998274</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>37.23531735231376</v>
+        <v>29.57807013660666</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.7295424941046468</v>
+        <v>0.1734991423423021</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L43" s="2" t="n">
         <v>0</v>
@@ -2743,31 +2743,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-0.8013859843286451</v>
+        <v>-0.0017859086290685</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>3071</v>
+        <v>3088</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>協禧</t>
+          <t>艾訊</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>791.0576214345724</v>
+        <v>791.5428041139836</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>33.6</v>
+        <v>144</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,13 +2778,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>57.80236994774686</v>
+        <v>61.03457006201996</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>28.40902040844198</v>
+        <v>37.23531735231376</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.7829829031135502</v>
+        <v>0.7295424941046468</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>3</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.0533375061689184</v>
+        <v>-0.8013859843286451</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>3059</v>
+        <v>3071</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>華晶科</t>
+          <t>協禧</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>789.0157793709948</v>
+        <v>791.0576214345724</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>49.35</v>
+        <v>33.6</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,16 +2831,16 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>61.30021418096327</v>
+        <v>57.80236994774686</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>35.72012135730295</v>
+        <v>28.40902040844198</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0.4943148480157628</v>
+        <v>0.7829829031135502</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.008391466478546401</v>
+        <v>-0.0533375061689184</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>2816</v>
+        <v>3031</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>旺旺保</t>
+          <t>佰鴻</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>783.6035697963395</v>
+        <v>787.3875374914686</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>33.8</v>
+        <v>30.5</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,16 +2884,16 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>57.18834130683078</v>
+        <v>53.76386823979556</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>29.93402887734022</v>
+        <v>11.79884198433533</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.6953733701336703</v>
+        <v>1.699794796885529</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-0.06544651189085531</v>
+        <v>-0.146352326645784</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, foreign_buy_3d, stronger_than_market, obv_uptrend, williams_r_recovery, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>2727</v>
+        <v>2816</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>王品</t>
+          <t>旺旺保</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>778.836950079756</v>
+        <v>783.6035697963395</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>246.5</v>
+        <v>33.8</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,16 +2937,16 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>64.02109501858556</v>
+        <v>57.18834130683078</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>37.028269582248</v>
+        <v>29.93402887734022</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.906134808441964</v>
+        <v>0.6953733701336703</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>0</v>
@@ -2955,11 +2955,11 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.1728406632683339</v>
+        <v>-0.06544651189085531</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -3018,21 +3018,21 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>3031</v>
+        <v>2457</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>佰鴻</t>
+          <t>飛宏</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>777.3875374914686</v>
+        <v>775.2721196522916</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>30.5</v>
+        <v>31.5</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>53.76386823979556</v>
+        <v>62.15428571163723</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>11.79884198433533</v>
+        <v>18.0744181517691</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>1.699794796885529</v>
+        <v>1.846930857078687</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-0.146352326645784</v>
+        <v>0.0559398827748864</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, foreign_buy_3d, stronger_than_market, obv_uptrend, williams_r_recovery, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, kd_golden_cross, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>2882</v>
+        <v>2727</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>國泰金</t>
+          <t>王品</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>766.3321383476655</v>
+        <v>768.836950079756</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>113</v>
+        <v>246.5</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,16 +3096,16 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>75.66146509642604</v>
+        <v>64.02109501858556</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>64.41481265367258</v>
+        <v>37.028269582248</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.6631325374097641</v>
+        <v>0.906134808441964</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>1.582020347069054</v>
+        <v>0.1728406632683339</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>2457</v>
+        <v>2882</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>飛宏</t>
+          <t>國泰金</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>765.2721196522916</v>
+        <v>766.3321383476655</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>31.5</v>
+        <v>113</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,16 +3149,16 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>62.15428571163723</v>
+        <v>75.66146509642604</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>18.0744181517691</v>
+        <v>64.41481265367258</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>1.846930857078687</v>
+        <v>0.6631325374097641</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.0559398827748864</v>
+        <v>1.582020347069054</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, kd_golden_cross, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>2897</v>
+        <v>2637</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>王道銀行</t>
+          <t>慧洋-KY</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>762.2454970840816</v>
+        <v>756.8259114955761</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>10.55</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,16 +3202,16 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>63.56835364939946</v>
+        <v>51.43798314765208</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>27.39407380184096</v>
+        <v>21.79905847225108</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.6061331864114746</v>
+        <v>0.3048749361647427</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.0294125062150242</v>
+        <v>-0.2665467230574807</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>2892</v>
+        <v>2636</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>第一金</t>
+          <t>台驊控股</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>758.3825083707203</v>
+        <v>756.8179788392748</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>32.3</v>
+        <v>70.7</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,49 +3255,49 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>74.94195406818562</v>
+        <v>61.56845391240681</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>35.24467074622799</v>
+        <v>22.27367431150912</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.7501098867873414</v>
+        <v>0.8917808232759518</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L53" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.3536778814534742</v>
+        <v>0.0170939238985824</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>2637</v>
+        <v>3048</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>慧洋-KY</t>
+          <t>益登</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>756.8259114955761</v>
+        <v>755.0932679602189</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>77.09999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,16 +3308,16 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>51.43798314765208</v>
+        <v>60.63656304127478</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>21.79905847225108</v>
+        <v>42.24357251301642</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.3048749361647427</v>
+        <v>0.4183228204379368</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-0.2665467230574807</v>
+        <v>-0.8883155523846638</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>2636</v>
+        <v>2897</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>台驊控股</t>
+          <t>王道銀行</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>756.8179788392748</v>
+        <v>752.2454970840816</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>70.7</v>
+        <v>10.55</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>61.56845391240681</v>
+        <v>63.56835364939946</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>22.27367431150912</v>
+        <v>27.39407380184096</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.8917808232759518</v>
+        <v>0.6061331864114746</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -3379,11 +3379,11 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.0170939238985824</v>
+        <v>0.0294125062150242</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -3495,21 +3495,21 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>2520</v>
+        <v>2892</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>冠德</t>
+          <t>第一金</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>748.0061832293318</v>
+        <v>748.3825083707203</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>34</v>
+        <v>32.3</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,49 +3520,49 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>55.61978191511314</v>
+        <v>74.94195406818562</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>34.38962795110628</v>
+        <v>35.24467074622799</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>1.858573276335954</v>
+        <v>0.7501098867873414</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M58" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.286949362079106</v>
+        <v>0.3536778814534742</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>2535</v>
+        <v>2520</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>達欣工</t>
+          <t>冠德</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>747.1777001302821</v>
+        <v>748.0061832293318</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>93.8</v>
+        <v>34</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>71.69860260967727</v>
+        <v>55.61978191511314</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>46.77395579973678</v>
+        <v>34.38962795110628</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.7118216609971789</v>
+        <v>1.858573276335954</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.7079061533780129</v>
+        <v>0.286949362079106</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>3048</v>
+        <v>2535</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>益登</t>
+          <t>達欣工</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>745.0932679602189</v>
+        <v>747.1777001302821</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>72.40000000000001</v>
+        <v>93.8</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,16 +3626,16 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>60.63656304127478</v>
+        <v>71.69860260967727</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>42.24357251301642</v>
+        <v>46.77395579973678</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.4183228204379368</v>
+        <v>0.7118216609971789</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>0</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.8883155523846638</v>
+        <v>0.7079061533780129</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3813,21 +3813,21 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>2464</v>
+        <v>3058</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>盟立</t>
+          <t>立德</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>740.6508987999962</v>
+        <v>744.0061397732821</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>173</v>
+        <v>9.65</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,16 +3838,16 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>59.000338751153</v>
+        <v>57.49200759845083</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>26.82966454559699</v>
+        <v>31.65957014218043</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>1.483265512847824</v>
+        <v>0.8014141611820413</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-1.286273077167479</v>
+        <v>0.0011257817141017</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, rsi_strong, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>2838</v>
+        <v>2495</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>聯邦銀</t>
+          <t>普安</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>735.5190230916337</v>
+        <v>741.8884517163502</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>22.4</v>
+        <v>52.1</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,16 +3891,16 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>66.08314326865099</v>
+        <v>59.66726412843772</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>31.98791552917001</v>
+        <v>30.96257875359367</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.8519023091633718</v>
+        <v>0.5210048917760662</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L65" s="2" t="n">
         <v>0</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.13748054749316</v>
+        <v>-0.0585735795975934</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3919,21 +3919,21 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>3058</v>
+        <v>2464</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>立德</t>
+          <t>盟立</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>734.0061397732821</v>
+        <v>740.6508987999962</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>9.65</v>
+        <v>173</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,16 +3944,16 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>57.49200759845083</v>
+        <v>59.000338751153</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>31.65957014218043</v>
+        <v>26.82966454559699</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.8014141611820413</v>
+        <v>1.483265512847824</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.0011257817141017</v>
+        <v>-1.286273077167479</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, rsi_strong, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>2495</v>
+        <v>2838</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>普安</t>
+          <t>聯邦銀</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>726.8884517163502</v>
+        <v>735.5190230916337</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>52.1</v>
+        <v>22.4</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,16 +3997,16 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>59.66726412843772</v>
+        <v>66.08314326865099</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>30.96257875359367</v>
+        <v>31.98791552917001</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.5210048917760662</v>
+        <v>0.8519023091633718</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L67" s="2" t="n">
         <v>0</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.0585735795975934</v>
+        <v>0.13748054749316</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4131,21 +4131,21 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>2484</v>
+        <v>3027</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>希華</t>
+          <t>盛達</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>716.9607096260137</v>
+        <v>709.0175831128928</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>66.90000000000001</v>
+        <v>21.55</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,16 +4156,16 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>63.02500821513865</v>
+        <v>57.90574624447615</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>43.83293302292265</v>
+        <v>24.95631024289385</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.6512124021496399</v>
+        <v>0.4487775017806309</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.7937145956668443</v>
+        <v>-0.005670584295878</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>2891</v>
+        <v>2820</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>中信金</t>
+          <t>華票</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>715.1169805925615</v>
+        <v>707.287191134571</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>70.5</v>
+        <v>17.75</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>67.86964694992528</v>
+        <v>67.6837135725404</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>59.13107792718174</v>
+        <v>31.23535443151544</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.8451668167726495</v>
+        <v>1.063652208223849</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.1949313180949392</v>
+        <v>0.0634874496833894</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>3027</v>
+        <v>2542</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>盛達</t>
+          <t>興富發</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>709.0175831128928</v>
+        <v>706.6892933829273</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>21.55</v>
+        <v>42.7</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,49 +4262,49 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>57.90574624447615</v>
+        <v>47.56087354508362</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>24.95631024289385</v>
+        <v>33.21352892926272</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.4487775017806309</v>
+        <v>1.231809679126046</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L72" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M72" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.005670584295878</v>
+        <v>-0.150450535253674</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>2820</v>
+        <v>2891</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>華票</t>
+          <t>中信金</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>707.287191134571</v>
+        <v>705.1169805925615</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>17.75</v>
+        <v>70.5</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>67.6837135725404</v>
+        <v>67.86964694992528</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>31.23535443151544</v>
+        <v>59.13107792718174</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>1.063652208223849</v>
+        <v>0.8451668167726495</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.0634874496833894</v>
+        <v>0.1949313180949392</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>2542</v>
+        <v>3033</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>興富發</t>
+          <t>威健</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>706.6892933829273</v>
+        <v>703.343007556615</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>42.7</v>
+        <v>51.2</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,49 +4368,49 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>47.56087354508362</v>
+        <v>60.82485457712686</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>33.21352892926272</v>
+        <v>32.49753704876098</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>1.231809679126046</v>
+        <v>0.9449810537717021</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L74" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M74" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.150450535253674</v>
+        <v>-0.4519607918165715</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>3037</v>
+        <v>2484</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>欣興</t>
+          <t>希華</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>697.8456525690829</v>
+        <v>701.9607096260137</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>1005</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,49 +4421,49 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>57.96253894217897</v>
+        <v>63.02500821513865</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>16.47044551877591</v>
+        <v>43.83293302292265</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>1.203091488654689</v>
+        <v>0.6512124021496399</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L75" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M75" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-4.429757634392342</v>
+        <v>0.7937145956668443</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, dealer_buy_3d, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>2547</v>
+        <v>3037</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>日勝生</t>
+          <t>欣興</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>695.6135826455167</v>
+        <v>697.8456525690829</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>10.95</v>
+        <v>1005</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,49 +4474,49 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>60.73006411768113</v>
+        <v>57.96253894217897</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>31.56837294621357</v>
+        <v>16.47044551877591</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.8206030538878106</v>
+        <v>1.203091488654689</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L76" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M76" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.0620669751945602</v>
+        <v>-4.429757634392342</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, dealer_buy_3d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>3033</v>
+        <v>2547</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>威健</t>
+          <t>日勝生</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>693.343007556615</v>
+        <v>695.6135826455167</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>51.2</v>
+        <v>10.95</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,16 +4527,16 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>60.82485457712686</v>
+        <v>60.73006411768113</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>32.49753704876098</v>
+        <v>31.56837294621357</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.9449810537717021</v>
+        <v>0.8206030538878106</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L77" s="2" t="n">
         <v>0</v>
@@ -4545,11 +4545,11 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.4519607918165715</v>
+        <v>0.0620669751945602</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -4661,21 +4661,21 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>2887</v>
+        <v>2739</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>台新新光金</t>
+          <t>寒舍</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>687.5616953877657</v>
+        <v>687.3632984710883</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>32.05</v>
+        <v>36.15</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,16 +4686,16 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>75.09936657585541</v>
+        <v>56.72909778275889</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>44.77972858535105</v>
+        <v>24.28969666254958</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.4005877672767888</v>
+        <v>1.090877640267621</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.4475366173771762</v>
+        <v>0.0181520305320413</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>2739</v>
+        <v>2546</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>寒舍</t>
+          <t>根基</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>687.3632984710883</v>
+        <v>687.3145145529074</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>36.15</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,16 +4739,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>56.72909778275889</v>
+        <v>59.6841050255204</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>24.28969666254958</v>
+        <v>35.95281952559054</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>1.090877640267621</v>
+        <v>1.25897844716014</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.0181520305320413</v>
+        <v>0.4569501219717549</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>2546</v>
+        <v>2460</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>根基</t>
+          <t>建通</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>687.3145145529074</v>
+        <v>683.7532814168118</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>93.40000000000001</v>
+        <v>35.05</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,16 +4792,16 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>59.6841050255204</v>
+        <v>57.47418029716412</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>35.95281952559054</v>
+        <v>15.30006595902026</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>1.25897844716014</v>
+        <v>1.234554933448039</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.4569501219717549</v>
+        <v>0.3695204227058073</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>2460</v>
+        <v>2476</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>建通</t>
+          <t>鉅祥</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>683.7532814168118</v>
+        <v>682.0744731140376</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>35.05</v>
+        <v>125.5</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,16 +4845,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>57.47418029716412</v>
+        <v>55.61302725637949</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>15.30006595902026</v>
+        <v>12.3298823306128</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>1.234554933448039</v>
+        <v>0.7781630354722606</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.3695204227058073</v>
+        <v>-0.126189587089792</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>2476</v>
+        <v>2515</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>鉅祥</t>
+          <t>中工</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>682.0744731140376</v>
+        <v>681.1342892817463</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>125.5</v>
+        <v>13.55</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,16 +4898,16 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>55.61302725637949</v>
+        <v>58.99674206606745</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>12.3298823306128</v>
+        <v>12.28854912365936</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.7781630354722606</v>
+        <v>1.333778260104673</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.126189587089792</v>
+        <v>0.0829403590301309</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, obv_uptrend, dealer_buy_3d, bb_squeeze_breakout, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>2515</v>
+        <v>2454</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>中工</t>
+          <t>聯發科</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>681.1342892817463</v>
+        <v>680.722357213241</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>13.55</v>
+        <v>4465</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,16 +4951,16 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>58.99674206606745</v>
+        <v>59.93901067283095</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>12.28854912365936</v>
+        <v>46.03982267533591</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>1.333778260104673</v>
+        <v>0.8142416932726272</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L85" s="2" t="n">
         <v>0</v>
@@ -4969,11 +4969,11 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.0829403590301309</v>
+        <v>-52.04709968814251</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, obv_uptrend, dealer_buy_3d, bb_squeeze_breakout, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, dealer_buy_3d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -5138,21 +5138,21 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>2454</v>
+        <v>2887</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>聯發科</t>
+          <t>台新新光金</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>670.722357213241</v>
+        <v>677.5616953877657</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>4465</v>
+        <v>32.05</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,16 +5163,16 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>59.93901067283095</v>
+        <v>75.09936657585541</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>46.03982267533591</v>
+        <v>44.77972858535105</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.8142416932726272</v>
+        <v>0.4005877672767888</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L89" s="2" t="n">
         <v>0</v>
@@ -5181,11 +5181,11 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-52.04709968814251</v>
+        <v>0.4475366173771762</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, dealer_buy_3d, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -5562,21 +5562,21 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>2610</v>
+        <v>2488</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>華航</t>
+          <t>漢平</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>632.2812512951473</v>
+        <v>631.7058397501817</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>21.8</v>
+        <v>54.8</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,49 +5587,49 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>71.37629465257646</v>
+        <v>64.30259932816486</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>37.04820462888487</v>
+        <v>24.89921683117728</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.7528256803684625</v>
+        <v>0.6512042845962132</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L97" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M97" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.2401159472823937</v>
+        <v>0.0667780239595912</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>2488</v>
+        <v>2910</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>漢平</t>
+          <t>統領</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>631.7058397501817</v>
+        <v>629.9748799243116</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>54.8</v>
+        <v>22.7</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,16 +5640,16 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>64.30259932816486</v>
+        <v>56.23907665960705</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>24.89921683117728</v>
+        <v>24.17459078837701</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.6512042845962132</v>
+        <v>0.2021385968848687</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>0</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.0667780239595912</v>
+        <v>0.1389540198038992</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5668,21 +5668,21 @@
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>2910</v>
+        <v>2610</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>統領</t>
+          <t>華航</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>629.9748799243116</v>
+        <v>622.2812512951473</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>22.7</v>
+        <v>21.8</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,29 +5693,29 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>56.23907665960705</v>
+        <v>71.37629465257646</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>24.17459078837701</v>
+        <v>37.04820462888487</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.2021385968848687</v>
+        <v>0.7528256803684625</v>
       </c>
       <c r="K99" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L99" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L99" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M99" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.1389540198038992</v>
+        <v>0.2401159472823937</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -6039,21 +6039,21 @@
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>3105</v>
+        <v>3042</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>穩懋</t>
+          <t>晶技</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>582.4098920668159</v>
+        <v>591.5858725532795</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>541</v>
+        <v>198</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,16 +6064,16 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>58.25502379381321</v>
+        <v>48.768632909944</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>14.61867667672193</v>
+        <v>31.41697220968627</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.932931916361133</v>
+        <v>1.181883579980067</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>3.023729281943233</v>
+        <v>-3.677268098186197</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>2812</v>
+        <v>3105</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>台中銀</t>
+          <t>穩懋</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>572.7346679943403</v>
+        <v>582.4098920668159</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>19.65</v>
+        <v>541</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,49 +6117,49 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>54.75603617057786</v>
+        <v>58.25502379381321</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>21.91058925919874</v>
+        <v>14.61867667672193</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.7132932513795547</v>
+        <v>0.932931916361133</v>
       </c>
       <c r="K107" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L107" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M107" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.1081618285085322</v>
+        <v>3.023729281943233</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, invest_trust_buy_2d, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>2701</v>
+        <v>2812</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>萬企</t>
+          <t>台中銀</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>568.1432908678861</v>
+        <v>572.7346679943403</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>10.6</v>
+        <v>19.65</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,49 +6170,49 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>58.08980457281207</v>
+        <v>54.75603617057786</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>24.06067949846758</v>
+        <v>21.91058925919874</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>1.229922994075598</v>
+        <v>0.7132932513795547</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L108" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M108" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.0342553708386433</v>
+        <v>0.1081618285085322</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, invest_trust_buy_2d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>2704</v>
+        <v>2701</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>國賓</t>
+          <t>萬企</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>567.9991474314035</v>
+        <v>568.1432908678861</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>46.1</v>
+        <v>10.6</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>71.37510000888805</v>
+        <v>58.08980457281207</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>38.20658883681141</v>
+        <v>24.06067949846758</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.5672205623185976</v>
+        <v>1.229922994075598</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>1</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.3842442536811529</v>
+        <v>0.0342553708386433</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>3003</v>
+        <v>2704</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>健和興</t>
+          <t>國賓</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>567.4792168547078</v>
+        <v>567.9991474314035</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>68.5</v>
+        <v>46.1</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,16 +6276,16 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>64.43951375548336</v>
+        <v>71.37510000888805</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>33.72491172908536</v>
+        <v>38.20658883681141</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>1.101443585150677</v>
+        <v>0.5672205623185976</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.3480036263213826</v>
+        <v>0.3842442536811529</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>2945</v>
+        <v>3003</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>三商家購</t>
+          <t>健和興</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>566.7377840236583</v>
+        <v>567.4792168547078</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>42.5</v>
+        <v>68.5</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>55.4194777567599</v>
+        <v>64.43951375548336</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>16.44269390356224</v>
+        <v>33.72491172908536</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.8326412557515963</v>
+        <v>1.101443585150677</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.1270926761265711</v>
+        <v>0.3480036263213826</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>3042</v>
+        <v>2945</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>晶技</t>
+          <t>三商家購</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>566.5858725532795</v>
+        <v>566.7377840236583</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>198</v>
+        <v>42.5</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>48.768632909944</v>
+        <v>55.4194777567599</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>31.41697220968627</v>
+        <v>16.44269390356224</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>1.181883579980067</v>
+        <v>0.8326412557515963</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-3.677268098186197</v>
+        <v>0.1270926761265711</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>2482</v>
+        <v>2474</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>連宇</t>
+          <t>可成</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>560.1439205090587</v>
+        <v>565.6990157809067</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>17.2</v>
+        <v>206</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,16 +6435,16 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>56.28289874879665</v>
+        <v>48.10188636621159</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>14.39655531793275</v>
+        <v>21.77904894851264</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>1.030245537019716</v>
+        <v>0.3626412534948771</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.0668676102649865</v>
+        <v>-2.212262677534248</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>2906</v>
+        <v>2482</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>高林</t>
+          <t>連宇</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>558.0494128781505</v>
+        <v>560.1439205090587</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>12.95</v>
+        <v>17.2</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,16 +6488,16 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>60.69686042809986</v>
+        <v>56.28289874879665</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>17.13748817710666</v>
+        <v>14.39655531793275</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.9655530744618122</v>
+        <v>1.030245537019716</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0371339706728613</v>
+        <v>0.0668676102649865</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>3051</v>
+        <v>2906</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>力特</t>
+          <t>高林</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>556.727351243786</v>
+        <v>558.0494128781505</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>27.9</v>
+        <v>12.95</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,16 +6541,16 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>53.63619513988222</v>
+        <v>60.69686042809986</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>14.89709385408612</v>
+        <v>17.13748817710666</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.4356163610900684</v>
+        <v>0.9655530744618122</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.1666143847103685</v>
+        <v>0.0371339706728613</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>2911</v>
+        <v>3051</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>麗嬰房</t>
+          <t>力特</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>552.1179775361458</v>
+        <v>556.727351243786</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>7.88</v>
+        <v>27.9</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,16 +6594,16 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>52.23183388765452</v>
+        <v>53.63619513988222</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>30.08019295124213</v>
+        <v>14.89709385408612</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.5835277296635493</v>
+        <v>0.4356163610900684</v>
       </c>
       <c r="K116" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.1743545914744737</v>
+        <v>-0.1666143847103685</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>2474</v>
+        <v>2911</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>可成</t>
+          <t>麗嬰房</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>550.6990157809067</v>
+        <v>552.1179775361458</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>206</v>
+        <v>7.88</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,16 +6647,16 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>48.10188636621159</v>
+        <v>52.23183388765452</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>21.77904894851264</v>
+        <v>30.08019295124213</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.3626412534948771</v>
+        <v>0.5835277296635493</v>
       </c>
       <c r="K117" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L117" s="2" t="n">
         <v>0</v>
@@ -6665,11 +6665,11 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-2.212262677534248</v>
+        <v>-0.1743545914744737</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -7470,21 +7470,21 @@
     </row>
     <row r="133">
       <c r="A133" s="2" t="n">
-        <v>3018</v>
+        <v>3017</v>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>隆銘綠能</t>
+          <t>奇鋐</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
         <v/>
       </c>
       <c r="D133" s="2" t="n">
-        <v>501.6915777300449</v>
+        <v>504.3427483043543</v>
       </c>
       <c r="E133" s="2" t="n">
-        <v>12</v>
+        <v>2420</v>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
@@ -7495,16 +7495,16 @@
         <v>0</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>61.70642937558908</v>
+        <v>45.56992939687098</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>14.94782138394188</v>
+        <v>19.15642168822882</v>
       </c>
       <c r="J133" s="2" t="n">
-        <v>2.083853783170389</v>
+        <v>0.6816832344225304</v>
       </c>
       <c r="K133" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L133" s="2" t="n">
         <v>0</v>
@@ -7513,31 +7513,31 @@
         <v>-1</v>
       </c>
       <c r="N133" s="2" t="n">
-        <v>0.0964691620543891</v>
+        <v>-25.94871045992824</v>
       </c>
       <c r="O133" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, volume_break, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n">
-        <v>3073</v>
+        <v>3018</v>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>天方能源</t>
+          <t>隆銘綠能</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
         <v/>
       </c>
       <c r="D134" s="2" t="n">
-        <v>499.2533069137605</v>
+        <v>501.6915777300449</v>
       </c>
       <c r="E134" s="2" t="n">
-        <v>22.05</v>
+        <v>12</v>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
@@ -7548,13 +7548,13 @@
         <v>0</v>
       </c>
       <c r="H134" s="2" t="n">
-        <v>54.05985868826023</v>
+        <v>61.70642937558908</v>
       </c>
       <c r="I134" s="2" t="n">
-        <v>16.1409631974169</v>
+        <v>14.94782138394188</v>
       </c>
       <c r="J134" s="2" t="n">
-        <v>1.621103107108869</v>
+        <v>2.083853783170389</v>
       </c>
       <c r="K134" s="2" t="n">
         <v>0</v>
@@ -7566,31 +7566,31 @@
         <v>-1</v>
       </c>
       <c r="N134" s="2" t="n">
-        <v>0.1677422193245082</v>
+        <v>0.0964691620543891</v>
       </c>
       <c r="O134" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>above_ema60, volume_break, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n">
-        <v>2536</v>
+        <v>3073</v>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>宏普</t>
+          <t>天方能源</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
         <v/>
       </c>
       <c r="D135" s="2" t="n">
-        <v>496.2911076989678</v>
+        <v>499.2533069137605</v>
       </c>
       <c r="E135" s="2" t="n">
-        <v>21.3</v>
+        <v>22.05</v>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
@@ -7601,13 +7601,13 @@
         <v>0</v>
       </c>
       <c r="H135" s="2" t="n">
-        <v>53.85860422076966</v>
+        <v>54.05985868826023</v>
       </c>
       <c r="I135" s="2" t="n">
-        <v>34.09981341175642</v>
+        <v>16.1409631974169</v>
       </c>
       <c r="J135" s="2" t="n">
-        <v>2.723724971747821</v>
+        <v>1.621103107108869</v>
       </c>
       <c r="K135" s="2" t="n">
         <v>0</v>
@@ -7619,31 +7619,31 @@
         <v>-1</v>
       </c>
       <c r="N135" s="2" t="n">
-        <v>0.1729984751472042</v>
+        <v>0.1677422193245082</v>
       </c>
       <c r="O135" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
-        <v>2538</v>
+        <v>2536</v>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>基泰</t>
+          <t>宏普</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
         <v/>
       </c>
       <c r="D136" s="2" t="n">
-        <v>495.2391146372631</v>
+        <v>496.2911076989678</v>
       </c>
       <c r="E136" s="2" t="n">
-        <v>10</v>
+        <v>21.3</v>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
@@ -7654,13 +7654,13 @@
         <v>0</v>
       </c>
       <c r="H136" s="2" t="n">
-        <v>54.2685100042051</v>
+        <v>53.85860422076966</v>
       </c>
       <c r="I136" s="2" t="n">
-        <v>32.78820775605379</v>
+        <v>34.09981341175642</v>
       </c>
       <c r="J136" s="2" t="n">
-        <v>0.986286735520712</v>
+        <v>2.723724971747821</v>
       </c>
       <c r="K136" s="2" t="n">
         <v>0</v>
@@ -7672,31 +7672,31 @@
         <v>-1</v>
       </c>
       <c r="N136" s="2" t="n">
-        <v>0.0252884323976665</v>
+        <v>0.1729984751472042</v>
       </c>
       <c r="O136" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n">
-        <v>3017</v>
+        <v>2538</v>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>奇鋐</t>
+          <t>基泰</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
         <v/>
       </c>
       <c r="D137" s="2" t="n">
-        <v>494.3427483043543</v>
+        <v>495.2391146372631</v>
       </c>
       <c r="E137" s="2" t="n">
-        <v>2420</v>
+        <v>10</v>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
@@ -7707,16 +7707,16 @@
         <v>0</v>
       </c>
       <c r="H137" s="2" t="n">
-        <v>45.56992939687098</v>
+        <v>54.2685100042051</v>
       </c>
       <c r="I137" s="2" t="n">
-        <v>19.15642168822882</v>
+        <v>32.78820775605379</v>
       </c>
       <c r="J137" s="2" t="n">
-        <v>0.6816832344225304</v>
+        <v>0.986286735520712</v>
       </c>
       <c r="K137" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L137" s="2" t="n">
         <v>0</v>
@@ -7725,11 +7725,11 @@
         <v>-1</v>
       </c>
       <c r="N137" s="2" t="n">
-        <v>-25.94871045992824</v>
+        <v>0.0252884323976665</v>
       </c>
       <c r="O137" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, dealer_buy_3d</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -9855,38 +9855,38 @@
     </row>
     <row r="178">
       <c r="A178" s="2" t="n">
-        <v>3036</v>
+        <v>2809</v>
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>文曄</t>
+          <t>京城銀</t>
         </is>
       </c>
       <c r="C178" s="2" t="n">
         <v/>
       </c>
       <c r="D178" s="2" t="n">
-        <v>366.3396773273247</v>
+        <v>360.0351332180986</v>
       </c>
       <c r="E178" s="2" t="n">
-        <v>225</v>
+        <v>34.2</v>
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="G178" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H178" s="2" t="n">
-        <v>34.84566988009962</v>
+        <v>20.05980282183059</v>
       </c>
       <c r="I178" s="2" t="n">
-        <v>34.53824928067135</v>
+        <v>43.43357050574636</v>
       </c>
       <c r="J178" s="2" t="n">
-        <v>1.101852725252135</v>
+        <v>0.3058439258734609</v>
       </c>
       <c r="K178" s="2" t="n">
         <v>0</v>
@@ -9898,7 +9898,7 @@
         <v>-1</v>
       </c>
       <c r="N178" s="2" t="n">
-        <v>-6.590959425701136</v>
+        <v>-2.656798760710905</v>
       </c>
       <c r="O178" s="2" t="inlineStr">
         <is>
@@ -9908,41 +9908,41 @@
     </row>
     <row r="179">
       <c r="A179" s="2" t="n">
-        <v>2809</v>
+        <v>2748</v>
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>京城銀</t>
+          <t>雲品</t>
         </is>
       </c>
       <c r="C179" s="2" t="n">
         <v/>
       </c>
       <c r="D179" s="2" t="n">
-        <v>360.0351332180986</v>
+        <v>358.7790261900394</v>
       </c>
       <c r="E179" s="2" t="n">
-        <v>34.2</v>
+        <v>40.25</v>
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G179" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H179" s="2" t="n">
-        <v>20.05980282183059</v>
+        <v>53.31701752360207</v>
       </c>
       <c r="I179" s="2" t="n">
-        <v>43.43357050574636</v>
+        <v>12.5907416217989</v>
       </c>
       <c r="J179" s="2" t="n">
-        <v>0.3058439258734609</v>
+        <v>0.7503775552887618</v>
       </c>
       <c r="K179" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L179" s="2" t="n">
         <v>0</v>
@@ -9951,31 +9951,31 @@
         <v>-1</v>
       </c>
       <c r="N179" s="2" t="n">
-        <v>-2.656798760710905</v>
+        <v>0.1119835029257513</v>
       </c>
       <c r="O179" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="n">
-        <v>2748</v>
+        <v>3036</v>
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>雲品</t>
+          <t>文曄</t>
         </is>
       </c>
       <c r="C180" s="2" t="n">
         <v/>
       </c>
       <c r="D180" s="2" t="n">
-        <v>358.7790261900394</v>
+        <v>356.3396773273247</v>
       </c>
       <c r="E180" s="2" t="n">
-        <v>40.25</v>
+        <v>225</v>
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
@@ -9986,16 +9986,16 @@
         <v>0</v>
       </c>
       <c r="H180" s="2" t="n">
-        <v>53.31701752360207</v>
+        <v>34.84566988009962</v>
       </c>
       <c r="I180" s="2" t="n">
-        <v>12.5907416217989</v>
+        <v>34.53824928067135</v>
       </c>
       <c r="J180" s="2" t="n">
-        <v>0.7503775552887618</v>
+        <v>1.101852725252135</v>
       </c>
       <c r="K180" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L180" s="2" t="n">
         <v>0</v>
@@ -10004,11 +10004,11 @@
         <v>-1</v>
       </c>
       <c r="N180" s="2" t="n">
-        <v>0.1119835029257513</v>
+        <v>-6.590959425701136</v>
       </c>
       <c r="O180" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>

</xml_diff>